<commit_message>
Add OpenAI CLIP prompt baseline results
</commit_message>
<xml_diff>
--- a/MMCL_OpenAI_CLIP_ViT-B16_Baselines.xlsx
+++ b/MMCL_OpenAI_CLIP_ViT-B16_Baselines.xlsx
@@ -1,159 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="14725"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="14725" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seed1993" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Seed1993" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="43">
-  <si>
-    <t>Method</t>
-  </si>
-  <si>
-    <t>Venue</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Aircraft B0 Inc10</t>
-  </si>
-  <si>
-    <t>Aircraft B50 Inc10</t>
-  </si>
-  <si>
-    <t>CIFAR100 B0 Inc10</t>
-  </si>
-  <si>
-    <t>CIFAR100 B50 Inc10</t>
-  </si>
-  <si>
-    <t>Cars B0 Inc10</t>
-  </si>
-  <si>
-    <t>Cars B50 Inc10</t>
-  </si>
-  <si>
-    <t>A_bar</t>
-  </si>
-  <si>
-    <t>A_B</t>
-  </si>
-  <si>
-    <t>ZS-CLIP</t>
-  </si>
-  <si>
-    <t>ICML</t>
-  </si>
-  <si>
-    <t>L2P</t>
-  </si>
-  <si>
-    <t>CVPR</t>
-  </si>
-  <si>
-    <t>DualPrompt</t>
-  </si>
-  <si>
-    <t>ECCV</t>
-  </si>
-  <si>
-    <t>CODA-Prompt</t>
-  </si>
-  <si>
-    <t>SimpleCIL</t>
-  </si>
-  <si>
-    <t>IJCV</t>
-  </si>
-  <si>
-    <t>PromptFusion</t>
-  </si>
-  <si>
-    <t>MoE-Adapters</t>
-  </si>
-  <si>
-    <t>RAPF</t>
-  </si>
-  <si>
-    <t>PROOF</t>
-  </si>
-  <si>
-    <t>TPAMI</t>
-  </si>
-  <si>
-    <t>ENGINE</t>
-  </si>
-  <si>
-    <t>ICCV</t>
-  </si>
-  <si>
-    <t>CLG-CBM</t>
-  </si>
-  <si>
-    <t>BOFA</t>
-  </si>
-  <si>
-    <t>AAAI</t>
-  </si>
-  <si>
-    <t>AREA</t>
-  </si>
-  <si>
-    <t>INR B0 Inc20</t>
-  </si>
-  <si>
-    <t>INR B100 Inc20</t>
-  </si>
-  <si>
-    <t>CUB B0 Inc20</t>
-  </si>
-  <si>
-    <t>CUB B100 Inc20</t>
-  </si>
-  <si>
-    <t>UCF B0 Inc10</t>
-  </si>
-  <si>
-    <t>UCF B50 Inc10</t>
-  </si>
-  <si>
-    <t>SUN B0 Inc30</t>
-  </si>
-  <si>
-    <t>SUN B150 Inc30</t>
-  </si>
-  <si>
-    <t>Food B0 Inc10</t>
-  </si>
-  <si>
-    <t>Food B50 Inc10</t>
-  </si>
-  <si>
-    <t>ObjectNet B0 Inc20</t>
-  </si>
-  <si>
-    <t>ObjectNet B100 Inc20</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ " numFmtId="164"/>
-    <numFmt formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ " numFmtId="165"/>
-    <numFmt formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ " numFmtId="166"/>
-    <numFmt formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ " numFmtId="167"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -516,7 +382,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -650,238 +516,318 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="50">
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="5" numFmtId="164">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="5" numFmtId="165">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="5" numFmtId="166">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="5" numFmtId="167">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="6" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="7" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="3" fillId="4" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="8" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="4" fillId="0" fontId="11" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="4" fillId="0" fontId="12" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="5" fillId="0" fontId="13" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="13" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="6" fillId="5" fontId="14" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="7" fillId="6" fontId="15" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="6" fillId="6" fontId="16" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="8" fillId="7" fontId="17" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="9" fillId="0" fontId="18" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="10" fillId="0" fontId="19" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="8" fontId="20" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="9" fontId="21" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="10" fontId="22" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="11" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="12" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="13" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="14" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="15" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="16" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="17" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="18" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="19" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="20" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="21" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="22" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="23" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="24" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="25" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="26" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="27" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="28" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="29" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="30" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="31" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="32" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="33" fontId="5" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="34" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49"/>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="49"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="0" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="0" fontId="3" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="2" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="50">
-    <cellStyle builtinId="0" name="常规" xfId="0"/>
-    <cellStyle builtinId="3" name="千位分隔" xfId="1"/>
-    <cellStyle builtinId="4" name="货币" xfId="2"/>
-    <cellStyle builtinId="5" name="百分比" xfId="3"/>
-    <cellStyle builtinId="6" name="千位分隔[0]" xfId="4"/>
-    <cellStyle builtinId="7" name="货币[0]" xfId="5"/>
-    <cellStyle builtinId="8" name="超链接" xfId="6"/>
-    <cellStyle builtinId="9" name="已访问的超链接" xfId="7"/>
-    <cellStyle builtinId="10" name="注释" xfId="8"/>
-    <cellStyle builtinId="11" name="警告文本" xfId="9"/>
-    <cellStyle builtinId="15" name="标题" xfId="10"/>
-    <cellStyle builtinId="53" name="解释性文本" xfId="11"/>
-    <cellStyle builtinId="16" name="标题 1" xfId="12"/>
-    <cellStyle builtinId="17" name="标题 2" xfId="13"/>
-    <cellStyle builtinId="18" name="标题 3" xfId="14"/>
-    <cellStyle builtinId="19" name="标题 4" xfId="15"/>
-    <cellStyle builtinId="20" name="输入" xfId="16"/>
-    <cellStyle builtinId="21" name="输出" xfId="17"/>
-    <cellStyle builtinId="22" name="计算" xfId="18"/>
-    <cellStyle builtinId="23" name="检查单元格" xfId="19"/>
-    <cellStyle builtinId="24" name="链接单元格" xfId="20"/>
-    <cellStyle builtinId="25" name="汇总" xfId="21"/>
-    <cellStyle builtinId="26" name="好" xfId="22"/>
-    <cellStyle builtinId="27" name="差" xfId="23"/>
-    <cellStyle builtinId="28" name="适中" xfId="24"/>
-    <cellStyle builtinId="29" name="强调文字颜色 1" xfId="25"/>
-    <cellStyle builtinId="30" name="20% - 强调文字颜色 1" xfId="26"/>
-    <cellStyle builtinId="31" name="40% - 强调文字颜色 1" xfId="27"/>
-    <cellStyle builtinId="32" name="60% - 强调文字颜色 1" xfId="28"/>
-    <cellStyle builtinId="33" name="强调文字颜色 2" xfId="29"/>
-    <cellStyle builtinId="34" name="20% - 强调文字颜色 2" xfId="30"/>
-    <cellStyle builtinId="35" name="40% - 强调文字颜色 2" xfId="31"/>
-    <cellStyle builtinId="36" name="60% - 强调文字颜色 2" xfId="32"/>
-    <cellStyle builtinId="37" name="强调文字颜色 3" xfId="33"/>
-    <cellStyle builtinId="38" name="20% - 强调文字颜色 3" xfId="34"/>
-    <cellStyle builtinId="39" name="40% - 强调文字颜色 3" xfId="35"/>
-    <cellStyle builtinId="40" name="60% - 强调文字颜色 3" xfId="36"/>
-    <cellStyle builtinId="41" name="强调文字颜色 4" xfId="37"/>
-    <cellStyle builtinId="42" name="20% - 强调文字颜色 4" xfId="38"/>
-    <cellStyle builtinId="43" name="40% - 强调文字颜色 4" xfId="39"/>
-    <cellStyle builtinId="44" name="60% - 强调文字颜色 4" xfId="40"/>
-    <cellStyle builtinId="45" name="强调文字颜色 5" xfId="41"/>
-    <cellStyle builtinId="46" name="20% - 强调文字颜色 5" xfId="42"/>
-    <cellStyle builtinId="47" name="40% - 强调文字颜色 5" xfId="43"/>
-    <cellStyle builtinId="48" name="60% - 强调文字颜色 5" xfId="44"/>
-    <cellStyle builtinId="49" name="强调文字颜色 6" xfId="45"/>
-    <cellStyle builtinId="50" name="20% - 强调文字颜色 6" xfId="46"/>
-    <cellStyle builtinId="51" name="40% - 强调文字颜色 6" xfId="47"/>
-    <cellStyle builtinId="52" name="60% - 强调文字颜色 6" xfId="48"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
     <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="8">
@@ -981,14 +927,82 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="2" defaultPivotStyle="PivotStylePreset2_Accent1 1" defaultTableStyle="TableStylePreset3_Accent1">
-    <tableStyle count="7" name="TableStylePreset3_Accent1" pivot="0">
-      <tableStyleElement dxfId="0" type="firstColumnStripe"/>
+  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1 1">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle count="1" name="PivotStylePreset2_Accent1 1" table="0">
-      <tableStyleElement dxfId="7" type="pageFieldValues"/>
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="1">
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1145,87 +1159,142 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O49"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.1"/>
   <cols>
-    <col customWidth="1" max="1" min="1" style="1" width="16"/>
-    <col customWidth="1" max="2" min="2" style="1" width="12.2083333333333"/>
-    <col customWidth="1" max="3" min="3" style="1" width="9.28333333333333"/>
-    <col customWidth="1" max="15" min="4" style="1" width="11"/>
+    <col width="16" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12.2083333333333" customWidth="1" style="1" min="2" max="2"/>
+    <col width="9.28333333333333" customWidth="1" style="1" min="3" max="3"/>
+    <col width="11" customWidth="1" style="1" min="4" max="15"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="26" r="1" s="10" spans="1:15">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="22" r="2" s="10" spans="1:15">
-      <c r="D2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="20" r="3" s="10" spans="1:15">
-      <c r="A3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>12</v>
+    <row r="1" ht="26" customHeight="1" s="10">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Venue</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Aircraft B0 Inc10</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="n"/>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Aircraft B50 Inc10</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="n"/>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>CIFAR100 B0 Inc10</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="n"/>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>CIFAR100 B50 Inc10</t>
+        </is>
+      </c>
+      <c r="K1" s="11" t="n"/>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Cars B0 Inc10</t>
+        </is>
+      </c>
+      <c r="M1" s="11" t="n"/>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Cars B50 Inc10</t>
+        </is>
+      </c>
+      <c r="O1" s="11" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="10">
+      <c r="A2" s="12" t="n"/>
+      <c r="B2" s="12" t="n"/>
+      <c r="C2" s="12" t="n"/>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="10">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>ZS-CLIP</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
       </c>
       <c r="C3" s="4" t="n">
         <v>2021</v>
@@ -1267,81 +1336,169 @@
         <v>49.5</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="4" s="10" spans="1:15">
-      <c r="A4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>14</v>
+    <row r="4" ht="20" customHeight="1" s="10">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>L2P</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C4" s="4" t="n">
         <v>2022</v>
       </c>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="5" s="10" spans="1:15">
-      <c r="A5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>16</v>
+      <c r="D4" s="5" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>28.08</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>48.99</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>81.44</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>72.72</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>80.27</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>71.08</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>74.38</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>69.23</v>
+      </c>
+      <c r="O4" s="5" t="n">
+        <v>51.8</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" s="10">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>DualPrompt</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
       </c>
       <c r="C5" s="4" t="n">
         <v>2022</v>
       </c>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="6" s="10" spans="1:15">
-      <c r="A6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>14</v>
+      <c r="D5" s="5" t="n">
+        <v>43.57</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>28.14</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>43.52</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>32.04</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>83.81</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>74.43000000000001</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>68.16</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>69.69</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>66.61</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" s="10">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CODA-Prompt</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C6" s="4" t="n">
         <v>2023</v>
       </c>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="7" s="10" spans="1:15">
-      <c r="A7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>19</v>
+      <c r="D6" s="5" t="n">
+        <v>38.42</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>23.07</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>25.23</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>76.53</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>62.19</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>71.23999999999999</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>57.97</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>66.17</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>49.33</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>62.17</v>
+      </c>
+      <c r="O6" s="5" t="n">
+        <v>44.72</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" s="10">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>SimpleCIL</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>IJCV</t>
+        </is>
       </c>
       <c r="C7" s="4" t="n">
         <v>2024</v>
@@ -1383,12 +1540,16 @@
         <v>68.33</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="8" s="10" spans="1:15">
-      <c r="A8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>16</v>
+    <row r="8" ht="20" customHeight="1" s="10">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>PromptFusion</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
       </c>
       <c r="C8" s="4" t="n">
         <v>2024</v>
@@ -1406,12 +1567,16 @@
       <c r="N8" s="5" t="n"/>
       <c r="O8" s="5" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="9" s="10" spans="1:15">
-      <c r="A9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>14</v>
+    <row r="9" ht="20" customHeight="1" s="10">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>MoE-Adapters</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C9" s="4" t="n">
         <v>2024</v>
@@ -1429,12 +1594,16 @@
       <c r="N9" s="5" t="n"/>
       <c r="O9" s="5" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="10" s="10" spans="1:15">
-      <c r="A10" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>16</v>
+    <row r="10" ht="20" customHeight="1" s="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>RAPF</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
       </c>
       <c r="C10" s="4" t="n">
         <v>2024</v>
@@ -1476,35 +1645,67 @@
         <v>52.63</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="11" s="10" spans="1:15">
-      <c r="A11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>24</v>
+    <row r="11" ht="20" customHeight="1" s="10">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>PROOF</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>TPAMI</t>
+        </is>
       </c>
       <c r="C11" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
-      <c r="N11" s="5" t="n"/>
-      <c r="O11" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="12" s="10" spans="1:15">
-      <c r="A12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>26</v>
+      <c r="D11" s="5" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>50.32</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>57.43</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>53.44</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>81.62</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>74.22</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>78.42</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>74.29000000000001</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>85.54000000000001</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>78.42</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>79.67</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" s="10">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>ICCV</t>
+        </is>
       </c>
       <c r="C12" s="4" t="n">
         <v>2025</v>
@@ -1546,12 +1747,16 @@
         <v>77.95999999999999</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="13" s="10" spans="1:15">
-      <c r="A13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>14</v>
+    <row r="13" ht="20" customHeight="1" s="10">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>CLG-CBM</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C13" s="4" t="n">
         <v>2025</v>
@@ -1593,12 +1798,16 @@
         <v>78.08</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="14" s="10" spans="1:15">
-      <c r="A14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>29</v>
+    <row r="14" ht="20" customHeight="1" s="10">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>BOFA</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
       </c>
       <c r="C14" s="4" t="n">
         <v>2026</v>
@@ -1640,12 +1849,16 @@
         <v>82.51000000000001</v>
       </c>
     </row>
-    <row customHeight="1" ht="21" r="15" s="10" spans="1:15">
-      <c r="A15" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>12</v>
+    <row r="15" ht="21" customHeight="1" s="10">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>AREA</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
       </c>
       <c r="C15" s="6" t="n">
         <v>2026</v>
@@ -1663,7 +1876,7 @@
       <c r="N15" s="6" t="n"/>
       <c r="O15" s="7" t="n"/>
     </row>
-    <row customHeight="1" ht="22" r="16" s="10" spans="1:15">
+    <row r="16" ht="22" customHeight="1" s="10">
       <c r="A16" s="8" t="n"/>
       <c r="B16" s="6" t="n"/>
       <c r="C16" s="6" t="n"/>
@@ -1680,7 +1893,7 @@
       <c r="N16" s="6" t="n"/>
       <c r="O16" s="6" t="n"/>
     </row>
-    <row customHeight="1" ht="22" r="17" s="10" spans="1:15">
+    <row r="17" ht="22" customHeight="1" s="10">
       <c r="A17" s="8" t="n"/>
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="6" t="n"/>
@@ -1697,79 +1910,134 @@
       <c r="N17" s="6" t="n"/>
       <c r="O17" s="6" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="18" s="10" spans="1:15">
-      <c r="A18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="J18" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="L18" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="N18" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="20" r="19" s="10" spans="1:15">
-      <c r="D19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="N19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="O19" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="20" r="20" s="10" spans="1:15">
-      <c r="A20" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>12</v>
+    <row r="18" ht="20" customHeight="1" s="10">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Venue</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>INR B0 Inc20</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>INR B100 Inc20</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>CUB B0 Inc20</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="n"/>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>CUB B100 Inc20</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="n"/>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>UCF B0 Inc10</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="n"/>
+      <c r="N18" s="9" t="inlineStr">
+        <is>
+          <t>UCF B50 Inc10</t>
+        </is>
+      </c>
+      <c r="O18" s="13" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" s="10">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" s="10">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>ZS-CLIP</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
       </c>
       <c r="C20" s="4" t="n">
         <v>2021</v>
@@ -1811,81 +2079,169 @@
         <v>66.28</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="21" s="10" spans="1:15">
-      <c r="A21" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>14</v>
+    <row r="21" ht="20" customHeight="1" s="10">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>L2P</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C21" s="4" t="n">
         <v>2022</v>
       </c>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="n"/>
-      <c r="K21" s="5" t="n"/>
-      <c r="L21" s="5" t="n"/>
-      <c r="M21" s="5" t="n"/>
-      <c r="N21" s="5" t="n"/>
-      <c r="O21" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="22" s="10" spans="1:15">
-      <c r="A22" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>16</v>
+      <c r="D21" s="5" t="n">
+        <v>82.45999999999999</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>75.22</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>63.83</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>70.28</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>56.19</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>46.65</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="M21" s="5" t="n">
+        <v>80.18000000000001</v>
+      </c>
+      <c r="N21" s="5" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="O21" s="5" t="n">
+        <v>68.36</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" s="10">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>DualPrompt</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
       </c>
       <c r="C22" s="4" t="n">
         <v>2022</v>
       </c>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="n"/>
-      <c r="I22" s="5" t="n"/>
-      <c r="J22" s="5" t="n"/>
-      <c r="K22" s="5" t="n"/>
-      <c r="L22" s="5" t="n"/>
-      <c r="M22" s="5" t="n"/>
-      <c r="N22" s="5" t="n"/>
-      <c r="O22" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="23" s="10" spans="1:15">
-      <c r="A23" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>14</v>
+      <c r="D22" s="5" t="n">
+        <v>82.18000000000001</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>74.55</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>72.05</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>62.03</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>71.36</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>60.09</v>
+      </c>
+      <c r="J22" s="5" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="K22" s="5" t="n">
+        <v>52.08</v>
+      </c>
+      <c r="L22" s="5" t="n">
+        <v>89.41</v>
+      </c>
+      <c r="M22" s="5" t="n">
+        <v>81.95999999999999</v>
+      </c>
+      <c r="N22" s="5" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="O22" s="5" t="n">
+        <v>70.94</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" s="10">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>CODA-Prompt</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C23" s="4" t="n">
         <v>2023</v>
       </c>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="n"/>
-      <c r="K23" s="5" t="n"/>
-      <c r="L23" s="5" t="n"/>
-      <c r="M23" s="5" t="n"/>
-      <c r="N23" s="5" t="n"/>
-      <c r="O23" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="24" s="10" spans="1:15">
-      <c r="A24" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>19</v>
+      <c r="D23" s="5" t="n">
+        <v>79.88</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>70.28</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>66.58</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>53.85</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>40.12</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>58.71</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>40.03</v>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>83.81999999999999</v>
+      </c>
+      <c r="M23" s="5" t="n">
+        <v>73.81999999999999</v>
+      </c>
+      <c r="N23" s="5" t="n">
+        <v>73.47</v>
+      </c>
+      <c r="O23" s="5" t="n">
+        <v>56.69</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" s="10">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>SimpleCIL</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>IJCV</t>
+        </is>
       </c>
       <c r="C24" s="4" t="n">
         <v>2024</v>
@@ -1927,12 +2283,16 @@
         <v>83.63</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="25" s="10" spans="1:15">
-      <c r="A25" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>16</v>
+    <row r="25" ht="20" customHeight="1" s="10">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>RAPF</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
       </c>
       <c r="C25" s="4" t="n">
         <v>2024</v>
@@ -1974,12 +2334,16 @@
         <v>80.79000000000001</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="26" s="10" spans="1:15">
-      <c r="A26" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>16</v>
+    <row r="26" ht="20" customHeight="1" s="10">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>PromptFusion</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
       </c>
       <c r="C26" s="4" t="n">
         <v>2024</v>
@@ -1997,12 +2361,16 @@
       <c r="N26" s="5" t="n"/>
       <c r="O26" s="5" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="27" s="10" spans="1:15">
-      <c r="A27" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>14</v>
+    <row r="27" ht="20" customHeight="1" s="10">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>MoE-Adapters</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C27" s="4" t="n">
         <v>2024</v>
@@ -2020,35 +2388,67 @@
       <c r="N27" s="5" t="n"/>
       <c r="O27" s="5" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="28" s="10" spans="1:15">
-      <c r="A28" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>24</v>
+    <row r="28" ht="20" customHeight="1" s="10">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>PROOF</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>TPAMI</t>
+        </is>
       </c>
       <c r="C28" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
-      <c r="K28" s="5" t="n"/>
-      <c r="L28" s="5" t="n"/>
-      <c r="M28" s="5" t="n"/>
-      <c r="N28" s="5" t="n"/>
-      <c r="O28" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="29" s="10" spans="1:15">
-      <c r="A29" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>26</v>
+      <c r="D28" s="5" t="n">
+        <v>80.91</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>75.28</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>81.37</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>75.83</v>
+      </c>
+      <c r="J28" s="5" t="n">
+        <v>77.52</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>75.19</v>
+      </c>
+      <c r="L28" s="5" t="n">
+        <v>93.36</v>
+      </c>
+      <c r="M28" s="5" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="N28" s="5" t="n">
+        <v>93.31</v>
+      </c>
+      <c r="O28" s="5" t="n">
+        <v>90.48999999999999</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1" s="10">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>ICCV</t>
+        </is>
       </c>
       <c r="C29" s="4" t="n">
         <v>2025</v>
@@ -2090,12 +2490,16 @@
         <v>89.5</v>
       </c>
     </row>
-    <row customHeight="1" ht="22" r="30" s="10" spans="1:15">
-      <c r="A30" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>14</v>
+    <row r="30" ht="22" customHeight="1" s="10">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>CLG-CBM</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C30" s="4" t="n">
         <v>2025</v>
@@ -2137,12 +2541,16 @@
         <v>92.31</v>
       </c>
     </row>
-    <row customHeight="1" ht="26" r="31" s="10" spans="1:15">
-      <c r="A31" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>29</v>
+    <row r="31" ht="26" customHeight="1" s="10">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>BOFA</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
       </c>
       <c r="C31" s="4" t="n">
         <v>2026</v>
@@ -2184,12 +2592,16 @@
         <v>89.16</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="32" s="10" spans="1:15">
-      <c r="A32" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>12</v>
+    <row r="32" ht="20" customHeight="1" s="10">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>AREA</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
       </c>
       <c r="C32" s="6" t="n">
         <v>2026</v>
@@ -2207,81 +2619,136 @@
       <c r="N32" s="6" t="n"/>
       <c r="O32" s="6" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="33" s="10" spans="1:15"/>
-    <row customHeight="1" ht="20" r="34" s="10" spans="1:15"/>
-    <row customHeight="1" ht="20" r="35" s="10" spans="1:15">
-      <c r="A35" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="J35" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="L35" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="N35" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="20" r="36" s="10" spans="1:15">
-      <c r="D36" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K36" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L36" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="M36" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="N36" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="O36" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="20" r="37" s="10" spans="1:15">
-      <c r="A37" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>12</v>
+    <row r="33" ht="20" customHeight="1" s="10"/>
+    <row r="34" ht="20" customHeight="1" s="10"/>
+    <row r="35" ht="20" customHeight="1" s="10">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Venue</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>SUN B0 Inc30</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>SUN B150 Inc30</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="n"/>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>Food B0 Inc10</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="n"/>
+      <c r="J35" s="9" t="inlineStr">
+        <is>
+          <t>Food B50 Inc10</t>
+        </is>
+      </c>
+      <c r="K35" s="13" t="n"/>
+      <c r="L35" s="9" t="inlineStr">
+        <is>
+          <t>ObjectNet B0 Inc20</t>
+        </is>
+      </c>
+      <c r="M35" s="13" t="n"/>
+      <c r="N35" s="9" t="inlineStr">
+        <is>
+          <t>ObjectNet B100 Inc20</t>
+        </is>
+      </c>
+      <c r="O35" s="13" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1" s="10">
+      <c r="A36" s="12" t="n"/>
+      <c r="B36" s="12" t="n"/>
+      <c r="C36" s="12" t="n"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+      <c r="N36" s="3" t="inlineStr">
+        <is>
+          <t>A_bar</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>A_B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1" s="10">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>ZS-CLIP</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
       </c>
       <c r="C37" s="4" t="n">
         <v>2021</v>
@@ -2323,81 +2790,169 @@
         <v>32.17</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="38" s="10" spans="1:15">
-      <c r="A38" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>14</v>
+    <row r="38" ht="20" customHeight="1" s="10">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>L2P</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C38" s="4" t="n">
         <v>2022</v>
       </c>
-      <c r="D38" s="5" t="n"/>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38" s="5" t="n"/>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="5" t="n"/>
-      <c r="I38" s="5" t="n"/>
-      <c r="J38" s="5" t="n"/>
-      <c r="K38" s="5" t="n"/>
-      <c r="L38" s="5" t="n"/>
-      <c r="M38" s="5" t="n"/>
-      <c r="N38" s="5" t="n"/>
-      <c r="O38" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="39" s="10" spans="1:15">
-      <c r="A39" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>16</v>
+      <c r="D38" s="5" t="n">
+        <v>80.34</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>70.55</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>65.66</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>86.26000000000001</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>77.53</v>
+      </c>
+      <c r="J38" s="5" t="n">
+        <v>83.48</v>
+      </c>
+      <c r="K38" s="5" t="n">
+        <v>76.38</v>
+      </c>
+      <c r="L38" s="5" t="n">
+        <v>61.88</v>
+      </c>
+      <c r="M38" s="5" t="n">
+        <v>47.92</v>
+      </c>
+      <c r="N38" s="5" t="n">
+        <v>55.97</v>
+      </c>
+      <c r="O38" s="5" t="n">
+        <v>44.89</v>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1" s="10">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>DualPrompt</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
       </c>
       <c r="C39" s="4" t="n">
         <v>2022</v>
       </c>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="5" t="n"/>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="5" t="n"/>
-      <c r="K39" s="5" t="n"/>
-      <c r="L39" s="5" t="n"/>
-      <c r="M39" s="5" t="n"/>
-      <c r="N39" s="5" t="n"/>
-      <c r="O39" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="40" s="10" spans="1:15">
-      <c r="A40" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>14</v>
+      <c r="D39" s="5" t="n">
+        <v>84.09999999999999</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>75.08</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>75.77</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>64.97</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>89.58</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>83.06999999999999</v>
+      </c>
+      <c r="J39" s="5" t="n">
+        <v>82.18000000000001</v>
+      </c>
+      <c r="K39" s="5" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="L39" s="5" t="n">
+        <v>60.73</v>
+      </c>
+      <c r="M39" s="5" t="n">
+        <v>48.23</v>
+      </c>
+      <c r="N39" s="5" t="n">
+        <v>54.06</v>
+      </c>
+      <c r="O39" s="5" t="n">
+        <v>43.32</v>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1" s="10">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>CODA-Prompt</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C40" s="4" t="n">
         <v>2023</v>
       </c>
-      <c r="D40" s="5" t="n"/>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="5" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="5" t="n"/>
-      <c r="I40" s="5" t="n"/>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="5" t="n"/>
-      <c r="L40" s="5" t="n"/>
-      <c r="M40" s="5" t="n"/>
-      <c r="N40" s="5" t="n"/>
-      <c r="O40" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="20" r="41" s="10" spans="1:15">
-      <c r="A41" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>19</v>
+      <c r="D40" s="5" t="n">
+        <v>79.36</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>69.06</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>69.31</v>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>56.58</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>76.84999999999999</v>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>60.01</v>
+      </c>
+      <c r="J40" s="5" t="n">
+        <v>71.23</v>
+      </c>
+      <c r="K40" s="5" t="n">
+        <v>53.83</v>
+      </c>
+      <c r="L40" s="5" t="n">
+        <v>61.19</v>
+      </c>
+      <c r="M40" s="5" t="n">
+        <v>47.96</v>
+      </c>
+      <c r="N40" s="5" t="n">
+        <v>50.42</v>
+      </c>
+      <c r="O40" s="5" t="n">
+        <v>37.3</v>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1" s="10">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>SimpleCIL</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>IJCV</t>
+        </is>
       </c>
       <c r="C41" s="4" t="n">
         <v>2024</v>
@@ -2439,12 +2994,16 @@
         <v>40.45</v>
       </c>
     </row>
-    <row customHeight="1" ht="17.55" r="42" s="10" spans="1:15">
-      <c r="A42" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>16</v>
+    <row r="42" ht="17.55" customHeight="1" s="10">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>RAPF</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
       </c>
       <c r="C42" s="4" t="n">
         <v>2024</v>
@@ -2486,12 +3045,16 @@
         <v>39.42</v>
       </c>
     </row>
-    <row customHeight="1" ht="17.55" r="43" s="10" spans="1:15">
-      <c r="A43" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>16</v>
+    <row r="43" ht="17.55" customHeight="1" s="10">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>PromptFusion</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
       </c>
       <c r="C43" s="4" t="n">
         <v>2024</v>
@@ -2509,12 +3072,16 @@
       <c r="N43" s="5" t="n"/>
       <c r="O43" s="5" t="n"/>
     </row>
-    <row customHeight="1" ht="17.55" r="44" s="10" spans="1:15">
-      <c r="A44" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>14</v>
+    <row r="44" ht="17.55" customHeight="1" s="10">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>MoE-Adapters</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C44" s="4" t="n">
         <v>2024</v>
@@ -2532,35 +3099,67 @@
       <c r="N44" s="5" t="n"/>
       <c r="O44" s="5" t="n"/>
     </row>
-    <row customHeight="1" ht="17.55" r="45" s="10" spans="1:15">
-      <c r="A45" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>24</v>
+    <row r="45" ht="17.55" customHeight="1" s="10">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>PROOF</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>TPAMI</t>
+        </is>
       </c>
       <c r="C45" s="4" t="n">
         <v>2025</v>
       </c>
-      <c r="D45" s="5" t="n"/>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="5" t="n"/>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="5" t="n"/>
-      <c r="I45" s="5" t="n"/>
-      <c r="J45" s="5" t="n"/>
-      <c r="K45" s="5" t="n"/>
-      <c r="L45" s="5" t="n"/>
-      <c r="M45" s="5" t="n"/>
-      <c r="N45" s="5" t="n"/>
-      <c r="O45" s="5" t="n"/>
-    </row>
-    <row customHeight="1" ht="17.55" r="46" s="10" spans="1:15">
-      <c r="A46" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>26</v>
+      <c r="D45" s="5" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>75.59</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>79.09</v>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>74.77</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>87.65000000000001</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>80.37</v>
+      </c>
+      <c r="J45" s="5" t="n">
+        <v>84.06999999999999</v>
+      </c>
+      <c r="K45" s="5" t="n">
+        <v>79.94</v>
+      </c>
+      <c r="L45" s="5" t="n">
+        <v>58.48</v>
+      </c>
+      <c r="M45" s="5" t="n">
+        <v>46.03</v>
+      </c>
+      <c r="N45" s="5" t="n">
+        <v>52.81</v>
+      </c>
+      <c r="O45" s="5" t="n">
+        <v>46.41</v>
+      </c>
+    </row>
+    <row r="46" ht="17.55" customHeight="1" s="10">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ENGINE</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>ICCV</t>
+        </is>
       </c>
       <c r="C46" s="4" t="n">
         <v>2025</v>
@@ -2602,12 +3201,16 @@
         <v>44.49</v>
       </c>
     </row>
-    <row customHeight="1" ht="17.55" r="47" s="10" spans="1:15">
-      <c r="A47" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>14</v>
+    <row r="47" ht="17.55" customHeight="1" s="10">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>CLG-CBM</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
       </c>
       <c r="C47" s="4" t="n">
         <v>2025</v>
@@ -2649,12 +3252,16 @@
         <v>46.09</v>
       </c>
     </row>
-    <row customHeight="1" ht="17.55" r="48" s="10" spans="1:15">
-      <c r="A48" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>29</v>
+    <row r="48" ht="17.55" customHeight="1" s="10">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>BOFA</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
       </c>
       <c r="C48" s="4" t="n">
         <v>2026</v>
@@ -2696,12 +3303,16 @@
         <v>48.58</v>
       </c>
     </row>
-    <row customHeight="1" ht="17.55" r="49" s="10" spans="1:15">
-      <c r="A49" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>12</v>
+    <row r="49" ht="17.55" customHeight="1" s="10">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>AREA</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
       </c>
       <c r="C49" s="6" t="n">
         <v>2026</v>
@@ -2719,38 +3330,38 @@
       <c r="N49" s="5" t="n"/>
       <c r="O49" s="5" t="n"/>
     </row>
-    <row customHeight="1" ht="17.55" r="50" s="10" spans="1:15"/>
-    <row customHeight="1" ht="17.55" r="51" s="10" spans="1:15"/>
+    <row r="50" ht="17.55" customHeight="1" s="10"/>
+    <row r="51" ht="17.55" customHeight="1" s="10"/>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="N35:O35"/>
     <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="B18:B19"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="J1:K1"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="L35:M35"/>
     <mergeCell ref="L1:M1"/>
-    <mergeCell ref="N1:O1"/>
     <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="A35:A36"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="J18:K18"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="B35:B36"/>
     <mergeCell ref="D35:E35"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="L35:M35"/>
-    <mergeCell ref="N35:O35"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C35:C36"/>
   </mergeCells>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record OpenAI and OpenCLIP experiment results
</commit_message>
<xml_diff>
--- a/MMCL_OpenAI_CLIP_ViT-B16_Baselines.xlsx
+++ b/MMCL_OpenAI_CLIP_ViT-B16_Baselines.xlsx
@@ -1340,18 +1340,42 @@
       <c r="C3" s="21" t="n">
         <v>2021</v>
       </c>
-      <c r="D3" s="20" t="n"/>
-      <c r="E3" s="20" t="n"/>
-      <c r="F3" s="20" t="n"/>
-      <c r="G3" s="20" t="n"/>
-      <c r="H3" s="20" t="n"/>
-      <c r="I3" s="20" t="n"/>
-      <c r="J3" s="20" t="n"/>
-      <c r="K3" s="20" t="n"/>
-      <c r="L3" s="20" t="n"/>
-      <c r="M3" s="20" t="n"/>
-      <c r="N3" s="20" t="n"/>
-      <c r="O3" s="20" t="n"/>
+      <c r="D3" s="20" t="n">
+        <v>31.98</v>
+      </c>
+      <c r="E3" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="F3" s="20" t="n">
+        <v>22.61</v>
+      </c>
+      <c r="G3" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="H3" s="20" t="n">
+        <v>69.14</v>
+      </c>
+      <c r="I3" s="20" t="n">
+        <v>62.78</v>
+      </c>
+      <c r="J3" s="20" t="n">
+        <v>64.95999999999999</v>
+      </c>
+      <c r="K3" s="20" t="n">
+        <v>62.78</v>
+      </c>
+      <c r="L3" s="20" t="n">
+        <v>66.98999999999999</v>
+      </c>
+      <c r="M3" s="20" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="N3" s="20" t="n">
+        <v>57.89</v>
+      </c>
+      <c r="O3" s="20" t="n">
+        <v>49.4</v>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1" s="27">
       <c r="A4" s="21" t="inlineStr">
@@ -1367,18 +1391,42 @@
       <c r="C4" s="21" t="n">
         <v>2022</v>
       </c>
-      <c r="D4" s="20" t="n"/>
-      <c r="E4" s="20" t="n"/>
-      <c r="F4" s="20" t="n"/>
-      <c r="G4" s="20" t="n"/>
-      <c r="H4" s="20" t="n"/>
-      <c r="I4" s="20" t="n"/>
-      <c r="J4" s="20" t="n"/>
-      <c r="K4" s="20" t="n"/>
-      <c r="L4" s="20" t="n"/>
-      <c r="M4" s="20" t="n"/>
-      <c r="N4" s="20" t="n"/>
-      <c r="O4" s="20" t="n"/>
+      <c r="D4" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="E4" s="20" t="n">
+        <v>29.46</v>
+      </c>
+      <c r="F4" s="20" t="n">
+        <v>48.49</v>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="H4" s="20" t="n">
+        <v>79.78</v>
+      </c>
+      <c r="I4" s="20" t="n">
+        <v>72.41</v>
+      </c>
+      <c r="J4" s="20" t="n">
+        <v>78.48</v>
+      </c>
+      <c r="K4" s="20" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="L4" s="20" t="n">
+        <v>71.19</v>
+      </c>
+      <c r="M4" s="20" t="n">
+        <v>55.99</v>
+      </c>
+      <c r="N4" s="20" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="O4" s="20" t="n">
+        <v>52.58</v>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1" s="27">
       <c r="A5" s="21" t="inlineStr">
@@ -1394,18 +1442,42 @@
       <c r="C5" s="21" t="n">
         <v>2022</v>
       </c>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="20" t="n"/>
-      <c r="F5" s="20" t="n"/>
-      <c r="G5" s="20" t="n"/>
-      <c r="H5" s="20" t="n"/>
-      <c r="I5" s="20" t="n"/>
-      <c r="J5" s="20" t="n"/>
-      <c r="K5" s="20" t="n"/>
-      <c r="L5" s="20" t="n"/>
-      <c r="M5" s="20" t="n"/>
-      <c r="N5" s="20" t="n"/>
-      <c r="O5" s="20" t="n"/>
+      <c r="D5" s="20" t="n">
+        <v>42.95</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>30.42</v>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>31.89</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>82.88</v>
+      </c>
+      <c r="I5" s="20" t="n">
+        <v>75.73999999999999</v>
+      </c>
+      <c r="J5" s="20" t="n">
+        <v>76.42</v>
+      </c>
+      <c r="K5" s="20" t="n">
+        <v>67.41</v>
+      </c>
+      <c r="L5" s="20" t="n">
+        <v>68.19</v>
+      </c>
+      <c r="M5" s="20" t="n">
+        <v>51.82</v>
+      </c>
+      <c r="N5" s="20" t="n">
+        <v>69.23999999999999</v>
+      </c>
+      <c r="O5" s="20" t="n">
+        <v>52.12</v>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1" s="27">
       <c r="A6" s="21" t="inlineStr">
@@ -1421,18 +1493,42 @@
       <c r="C6" s="21" t="n">
         <v>2023</v>
       </c>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="20" t="n"/>
-      <c r="L6" s="20" t="n"/>
-      <c r="M6" s="20" t="n"/>
-      <c r="N6" s="20" t="n"/>
-      <c r="O6" s="20" t="n"/>
+      <c r="D6" s="20" t="n">
+        <v>40.33</v>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>26.31</v>
+      </c>
+      <c r="F6" s="20" t="n">
+        <v>42.42</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>75.75</v>
+      </c>
+      <c r="I6" s="20" t="n">
+        <v>64.73</v>
+      </c>
+      <c r="J6" s="20" t="n">
+        <v>68.15000000000001</v>
+      </c>
+      <c r="K6" s="20" t="n">
+        <v>55.71</v>
+      </c>
+      <c r="L6" s="20" t="n">
+        <v>62.15</v>
+      </c>
+      <c r="M6" s="20" t="n">
+        <v>47.61</v>
+      </c>
+      <c r="N6" s="20" t="n">
+        <v>64.27</v>
+      </c>
+      <c r="O6" s="20" t="n">
+        <v>44.38</v>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1" s="27">
       <c r="A7" s="21" t="inlineStr">
@@ -1448,18 +1544,42 @@
       <c r="C7" s="21" t="n">
         <v>2023</v>
       </c>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="20" t="n"/>
-      <c r="F7" s="20" t="n"/>
-      <c r="G7" s="20" t="n"/>
-      <c r="H7" s="20" t="n"/>
-      <c r="I7" s="20" t="n"/>
-      <c r="J7" s="20" t="n"/>
-      <c r="K7" s="20" t="n"/>
-      <c r="L7" s="20" t="n"/>
-      <c r="M7" s="20" t="n"/>
-      <c r="N7" s="20" t="n"/>
-      <c r="O7" s="20" t="n"/>
+      <c r="D7" s="20" t="n">
+        <v>65.61</v>
+      </c>
+      <c r="E7" s="20" t="n">
+        <v>58.09</v>
+      </c>
+      <c r="F7" s="20" t="n">
+        <v>62.55</v>
+      </c>
+      <c r="G7" s="20" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>89.63</v>
+      </c>
+      <c r="I7" s="20" t="n">
+        <v>84.72</v>
+      </c>
+      <c r="J7" s="20" t="n">
+        <v>86.31</v>
+      </c>
+      <c r="K7" s="20" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="L7" s="20" t="n">
+        <v>91.27</v>
+      </c>
+      <c r="M7" s="20" t="n">
+        <v>83.48999999999999</v>
+      </c>
+      <c r="N7" s="20" t="n">
+        <v>88.33</v>
+      </c>
+      <c r="O7" s="20" t="n">
+        <v>82.44</v>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1" s="27">
       <c r="A8" s="21" t="inlineStr">
@@ -1475,18 +1595,42 @@
       <c r="C8" s="21" t="n">
         <v>2023</v>
       </c>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="20" t="n"/>
-      <c r="I8" s="20" t="n"/>
-      <c r="J8" s="20" t="n"/>
-      <c r="K8" s="20" t="n"/>
-      <c r="L8" s="20" t="n"/>
-      <c r="M8" s="20" t="n"/>
-      <c r="N8" s="20" t="n"/>
-      <c r="O8" s="20" t="n"/>
+      <c r="D8" s="20" t="n">
+        <v>57.12</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>47.22</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>53.02</v>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>49.14</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>79.70999999999999</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>72.28</v>
+      </c>
+      <c r="J8" s="20" t="n">
+        <v>75.73</v>
+      </c>
+      <c r="K8" s="20" t="n">
+        <v>70.34</v>
+      </c>
+      <c r="L8" s="20" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="M8" s="20" t="n">
+        <v>72.23</v>
+      </c>
+      <c r="N8" s="20" t="n">
+        <v>80.63</v>
+      </c>
+      <c r="O8" s="20" t="n">
+        <v>75.12</v>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1" s="27">
       <c r="A9" s="21" t="inlineStr">
@@ -1502,18 +1646,42 @@
       <c r="C9" s="21" t="n">
         <v>2024</v>
       </c>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="20" t="n"/>
-      <c r="K9" s="20" t="n"/>
-      <c r="L9" s="20" t="n"/>
-      <c r="M9" s="20" t="n"/>
-      <c r="N9" s="20" t="n"/>
-      <c r="O9" s="20" t="n"/>
+      <c r="D9" s="20" t="n">
+        <v>53.62</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>43.02</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>46.94</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>43.02</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>65.98</v>
+      </c>
+      <c r="J9" s="20" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="K9" s="20" t="n">
+        <v>65.98</v>
+      </c>
+      <c r="L9" s="20" t="n">
+        <v>80.64</v>
+      </c>
+      <c r="M9" s="20" t="n">
+        <v>68.36</v>
+      </c>
+      <c r="N9" s="20" t="n">
+        <v>75.01000000000001</v>
+      </c>
+      <c r="O9" s="20" t="n">
+        <v>68.36</v>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1" s="27">
       <c r="A10" s="21" t="inlineStr">
@@ -1599,18 +1767,42 @@
       <c r="C12" s="21" t="n">
         <v>2024</v>
       </c>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="20" t="n"/>
-      <c r="I12" s="20" t="n"/>
-      <c r="J12" s="20" t="n"/>
-      <c r="K12" s="20" t="n"/>
-      <c r="L12" s="20" t="n"/>
-      <c r="M12" s="20" t="n"/>
-      <c r="N12" s="20" t="n"/>
-      <c r="O12" s="20" t="n"/>
+      <c r="D12" s="20" t="n">
+        <v>42.78</v>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>19.68</v>
+      </c>
+      <c r="F12" s="20" t="n">
+        <v>36.27</v>
+      </c>
+      <c r="G12" s="20" t="n">
+        <v>21.21</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <v>82.97</v>
+      </c>
+      <c r="I12" s="20" t="n">
+        <v>75.38</v>
+      </c>
+      <c r="J12" s="20" t="n">
+        <v>80.34</v>
+      </c>
+      <c r="K12" s="20" t="n">
+        <v>75.89</v>
+      </c>
+      <c r="L12" s="20" t="n">
+        <v>69.67</v>
+      </c>
+      <c r="M12" s="20" t="n">
+        <v>47.81</v>
+      </c>
+      <c r="N12" s="20" t="n">
+        <v>66.28</v>
+      </c>
+      <c r="O12" s="20" t="n">
+        <v>48.67</v>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1" s="27">
       <c r="A13" s="21" t="inlineStr">
@@ -1626,18 +1818,42 @@
       <c r="C13" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="20" t="n"/>
-      <c r="H13" s="20" t="n"/>
-      <c r="I13" s="20" t="n"/>
-      <c r="J13" s="20" t="n"/>
-      <c r="K13" s="20" t="n"/>
-      <c r="L13" s="20" t="n"/>
-      <c r="M13" s="20" t="n"/>
-      <c r="N13" s="20" t="n"/>
-      <c r="O13" s="20" t="n"/>
+      <c r="D13" s="20" t="n">
+        <v>58.19</v>
+      </c>
+      <c r="E13" s="20" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>56.47</v>
+      </c>
+      <c r="G13" s="20" t="n">
+        <v>52.93</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <v>79.70999999999999</v>
+      </c>
+      <c r="I13" s="20" t="n">
+        <v>73.63</v>
+      </c>
+      <c r="J13" s="20" t="n">
+        <v>77.42</v>
+      </c>
+      <c r="K13" s="20" t="n">
+        <v>73.47</v>
+      </c>
+      <c r="L13" s="20" t="n">
+        <v>87.17</v>
+      </c>
+      <c r="M13" s="20" t="n">
+        <v>78.89</v>
+      </c>
+      <c r="N13" s="20" t="n">
+        <v>83.56999999999999</v>
+      </c>
+      <c r="O13" s="20" t="n">
+        <v>79.52</v>
+      </c>
     </row>
     <row r="14" ht="20" customHeight="1" s="27">
       <c r="A14" s="21" t="inlineStr">
@@ -1704,18 +1920,42 @@
       <c r="C15" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="20" t="n"/>
-      <c r="I15" s="20" t="n"/>
-      <c r="J15" s="20" t="n"/>
-      <c r="K15" s="20" t="n"/>
-      <c r="L15" s="20" t="n"/>
-      <c r="M15" s="20" t="n"/>
-      <c r="N15" s="20" t="n"/>
-      <c r="O15" s="20" t="n"/>
+      <c r="D15" s="20" t="n">
+        <v>60.31</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>51.97</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="G15" s="20" t="n">
+        <v>49.44</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>81</v>
+      </c>
+      <c r="I15" s="20" t="n">
+        <v>74.69</v>
+      </c>
+      <c r="J15" s="20" t="n">
+        <v>75.73999999999999</v>
+      </c>
+      <c r="K15" s="20" t="n">
+        <v>73.73</v>
+      </c>
+      <c r="L15" s="20" t="n">
+        <v>86.03</v>
+      </c>
+      <c r="M15" s="20" t="n">
+        <v>78.06</v>
+      </c>
+      <c r="N15" s="20" t="n">
+        <v>78.92</v>
+      </c>
+      <c r="O15" s="20" t="n">
+        <v>77.81</v>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1" s="27">
       <c r="A16" s="21" t="inlineStr">
@@ -1782,18 +2022,42 @@
       <c r="C17" s="22" t="n">
         <v>2026</v>
       </c>
-      <c r="D17" s="22" t="n"/>
-      <c r="E17" s="23" t="n"/>
-      <c r="F17" s="22" t="n"/>
-      <c r="G17" s="23" t="n"/>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="23" t="n"/>
-      <c r="J17" s="22" t="n"/>
-      <c r="K17" s="23" t="n"/>
-      <c r="L17" s="22" t="n"/>
-      <c r="M17" s="23" t="n"/>
-      <c r="N17" s="22" t="n"/>
-      <c r="O17" s="23" t="n"/>
+      <c r="D17" s="22" t="n">
+        <v>63.89</v>
+      </c>
+      <c r="E17" s="23" t="n">
+        <v>54.43</v>
+      </c>
+      <c r="F17" s="22" t="n">
+        <v>59.72</v>
+      </c>
+      <c r="G17" s="23" t="n">
+        <v>55.24</v>
+      </c>
+      <c r="H17" s="22" t="n">
+        <v>80.91</v>
+      </c>
+      <c r="I17" s="23" t="n">
+        <v>75.75</v>
+      </c>
+      <c r="J17" s="22" t="n">
+        <v>76.70999999999999</v>
+      </c>
+      <c r="K17" s="23" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="L17" s="22" t="n">
+        <v>87.81999999999999</v>
+      </c>
+      <c r="M17" s="23" t="n">
+        <v>78.18000000000001</v>
+      </c>
+      <c r="N17" s="22" t="n">
+        <v>88.23999999999999</v>
+      </c>
+      <c r="O17" s="23" t="n">
+        <v>83.56999999999999</v>
+      </c>
     </row>
     <row r="18" ht="22" customHeight="1" s="27">
       <c r="A18" s="24" t="n"/>
@@ -1967,8 +2231,12 @@
       <c r="G22" s="20" t="n"/>
       <c r="H22" s="20" t="n"/>
       <c r="I22" s="20" t="n"/>
-      <c r="J22" s="20" t="n"/>
-      <c r="K22" s="20" t="n"/>
+      <c r="J22" s="20" t="n">
+        <v>53.23</v>
+      </c>
+      <c r="K22" s="20" t="n">
+        <v>47.58</v>
+      </c>
       <c r="L22" s="20" t="n"/>
       <c r="M22" s="20" t="n"/>
       <c r="N22" s="20" t="n"/>
@@ -1988,18 +2256,30 @@
       <c r="C23" s="21" t="n">
         <v>2022</v>
       </c>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="20" t="n"/>
-      <c r="F23" s="20" t="n"/>
-      <c r="G23" s="20" t="n"/>
+      <c r="D23" s="20" t="n">
+        <v>81.78</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>74.31999999999999</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <v>74.23</v>
+      </c>
+      <c r="G23" s="20" t="n">
+        <v>63.63</v>
+      </c>
       <c r="H23" s="20" t="n"/>
       <c r="I23" s="20" t="n"/>
       <c r="J23" s="20" t="n"/>
       <c r="K23" s="20" t="n"/>
       <c r="L23" s="20" t="n"/>
       <c r="M23" s="20" t="n"/>
-      <c r="N23" s="20" t="n"/>
-      <c r="O23" s="20" t="n"/>
+      <c r="N23" s="20" t="n">
+        <v>81</v>
+      </c>
+      <c r="O23" s="20" t="n">
+        <v>67.45</v>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1" s="27">
       <c r="A24" s="21" t="inlineStr">
@@ -2015,18 +2295,38 @@
       <c r="C24" s="21" t="n">
         <v>2022</v>
       </c>
-      <c r="D24" s="20" t="n"/>
-      <c r="E24" s="20" t="n"/>
-      <c r="F24" s="20" t="n"/>
-      <c r="G24" s="20" t="n"/>
+      <c r="D24" s="20" t="n">
+        <v>81.95999999999999</v>
+      </c>
+      <c r="E24" s="20" t="n">
+        <v>75.15000000000001</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <v>72.26000000000001</v>
+      </c>
+      <c r="G24" s="20" t="n">
+        <v>62.18</v>
+      </c>
       <c r="H24" s="20" t="n"/>
       <c r="I24" s="20" t="n"/>
-      <c r="J24" s="20" t="n"/>
-      <c r="K24" s="20" t="n"/>
-      <c r="L24" s="20" t="n"/>
-      <c r="M24" s="20" t="n"/>
-      <c r="N24" s="20" t="n"/>
-      <c r="O24" s="20" t="n"/>
+      <c r="J24" s="20" t="n">
+        <v>66.75</v>
+      </c>
+      <c r="K24" s="20" t="n">
+        <v>53.77</v>
+      </c>
+      <c r="L24" s="20" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="M24" s="20" t="n">
+        <v>82.19</v>
+      </c>
+      <c r="N24" s="20" t="n">
+        <v>81.42</v>
+      </c>
+      <c r="O24" s="20" t="n">
+        <v>69.91</v>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1" s="27">
       <c r="A25" s="21" t="inlineStr">
@@ -2044,16 +2344,32 @@
       </c>
       <c r="D25" s="20" t="n"/>
       <c r="E25" s="20" t="n"/>
-      <c r="F25" s="20" t="n"/>
-      <c r="G25" s="20" t="n"/>
-      <c r="H25" s="20" t="n"/>
-      <c r="I25" s="20" t="n"/>
-      <c r="J25" s="20" t="n"/>
-      <c r="K25" s="20" t="n"/>
+      <c r="F25" s="20" t="n">
+        <v>66.97</v>
+      </c>
+      <c r="G25" s="20" t="n">
+        <v>54.25</v>
+      </c>
+      <c r="H25" s="20" t="n">
+        <v>64</v>
+      </c>
+      <c r="I25" s="20" t="n">
+        <v>44.74</v>
+      </c>
+      <c r="J25" s="20" t="n">
+        <v>58.34</v>
+      </c>
+      <c r="K25" s="20" t="n">
+        <v>41.65</v>
+      </c>
       <c r="L25" s="20" t="n"/>
       <c r="M25" s="20" t="n"/>
-      <c r="N25" s="20" t="n"/>
-      <c r="O25" s="20" t="n"/>
+      <c r="N25" s="20" t="n">
+        <v>74.95999999999999</v>
+      </c>
+      <c r="O25" s="20" t="n">
+        <v>57.94</v>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1" s="27">
       <c r="A26" s="21" t="inlineStr">
@@ -2071,16 +2387,24 @@
       </c>
       <c r="D26" s="20" t="n"/>
       <c r="E26" s="20" t="n"/>
-      <c r="F26" s="20" t="n"/>
-      <c r="G26" s="20" t="n"/>
+      <c r="F26" s="20" t="n">
+        <v>82.06</v>
+      </c>
+      <c r="G26" s="20" t="n">
+        <v>79.97</v>
+      </c>
       <c r="H26" s="20" t="n"/>
       <c r="I26" s="20" t="n"/>
       <c r="J26" s="20" t="n"/>
       <c r="K26" s="20" t="n"/>
       <c r="L26" s="20" t="n"/>
       <c r="M26" s="20" t="n"/>
-      <c r="N26" s="20" t="n"/>
-      <c r="O26" s="20" t="n"/>
+      <c r="N26" s="20" t="n">
+        <v>66.05</v>
+      </c>
+      <c r="O26" s="20" t="n">
+        <v>98.11</v>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1" s="27">
       <c r="A27" s="21" t="inlineStr">
@@ -2098,12 +2422,24 @@
       </c>
       <c r="D27" s="20" t="n"/>
       <c r="E27" s="20" t="n"/>
-      <c r="F27" s="20" t="n"/>
-      <c r="G27" s="20" t="n"/>
-      <c r="H27" s="20" t="n"/>
-      <c r="I27" s="20" t="n"/>
-      <c r="J27" s="20" t="n"/>
-      <c r="K27" s="20" t="n"/>
+      <c r="F27" s="20" t="n">
+        <v>71</v>
+      </c>
+      <c r="G27" s="20" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="H27" s="20" t="n">
+        <v>82.79000000000001</v>
+      </c>
+      <c r="I27" s="20" t="n">
+        <v>75.31999999999999</v>
+      </c>
+      <c r="J27" s="20" t="n">
+        <v>81.91</v>
+      </c>
+      <c r="K27" s="20" t="n">
+        <v>78.37</v>
+      </c>
       <c r="L27" s="20" t="n"/>
       <c r="M27" s="20" t="n"/>
       <c r="N27" s="20" t="n"/>
@@ -2125,16 +2461,24 @@
       </c>
       <c r="D28" s="20" t="n"/>
       <c r="E28" s="20" t="n"/>
-      <c r="F28" s="20" t="n"/>
-      <c r="G28" s="20" t="n"/>
+      <c r="F28" s="20" t="n">
+        <v>71</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>67.93000000000001</v>
+      </c>
       <c r="H28" s="20" t="n"/>
       <c r="I28" s="20" t="n"/>
       <c r="J28" s="20" t="n"/>
       <c r="K28" s="20" t="n"/>
       <c r="L28" s="20" t="n"/>
       <c r="M28" s="20" t="n"/>
-      <c r="N28" s="20" t="n"/>
-      <c r="O28" s="20" t="n"/>
+      <c r="N28" s="20" t="n">
+        <v>87.22</v>
+      </c>
+      <c r="O28" s="20" t="n">
+        <v>83.59</v>
+      </c>
     </row>
     <row r="29" ht="20" customHeight="1" s="27">
       <c r="A29" s="21" t="inlineStr">
@@ -2156,8 +2500,12 @@
       <c r="G29" s="20" t="n"/>
       <c r="H29" s="20" t="n"/>
       <c r="I29" s="20" t="n"/>
-      <c r="J29" s="20" t="n"/>
-      <c r="K29" s="20" t="n"/>
+      <c r="J29" s="20" t="n">
+        <v>58.71</v>
+      </c>
+      <c r="K29" s="20" t="n">
+        <v>48.26</v>
+      </c>
       <c r="L29" s="20" t="n"/>
       <c r="M29" s="20" t="n"/>
       <c r="N29" s="20" t="n"/>
@@ -2265,8 +2613,12 @@
       <c r="G32" s="20" t="n"/>
       <c r="H32" s="20" t="n"/>
       <c r="I32" s="20" t="n"/>
-      <c r="J32" s="20" t="n"/>
-      <c r="K32" s="20" t="n"/>
+      <c r="J32" s="20" t="n">
+        <v>79.03</v>
+      </c>
+      <c r="K32" s="20" t="n">
+        <v>75.48999999999999</v>
+      </c>
       <c r="L32" s="20" t="n"/>
       <c r="M32" s="20" t="n"/>
       <c r="N32" s="20" t="n"/>
@@ -2286,10 +2638,18 @@
       <c r="C33" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="D33" s="20" t="n"/>
-      <c r="E33" s="20" t="n"/>
-      <c r="F33" s="20" t="n"/>
-      <c r="G33" s="20" t="n"/>
+      <c r="D33" s="20" t="n">
+        <v>83.48</v>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>77.42</v>
+      </c>
+      <c r="F33" s="20" t="n">
+        <v>80.16</v>
+      </c>
+      <c r="G33" s="20" t="n">
+        <v>77.48</v>
+      </c>
       <c r="H33" s="20" t="n">
         <v>85.12</v>
       </c>
@@ -2302,10 +2662,18 @@
       <c r="K33" s="20" t="n">
         <v>76</v>
       </c>
-      <c r="L33" s="20" t="n"/>
-      <c r="M33" s="20" t="n"/>
-      <c r="N33" s="20" t="n"/>
-      <c r="O33" s="20" t="n"/>
+      <c r="L33" s="20" t="n">
+        <v>94.88</v>
+      </c>
+      <c r="M33" s="20" t="n">
+        <v>90.06999999999999</v>
+      </c>
+      <c r="N33" s="20" t="n">
+        <v>92.52</v>
+      </c>
+      <c r="O33" s="20" t="n">
+        <v>89.16</v>
+      </c>
     </row>
     <row r="34" ht="22" customHeight="1" s="27">
       <c r="A34" s="21" t="inlineStr">
@@ -2321,18 +2689,38 @@
       <c r="C34" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="D34" s="20" t="n"/>
-      <c r="E34" s="20" t="n"/>
-      <c r="F34" s="20" t="n"/>
-      <c r="G34" s="20" t="n"/>
+      <c r="D34" s="20" t="n">
+        <v>81.92</v>
+      </c>
+      <c r="E34" s="20" t="n">
+        <v>76.62</v>
+      </c>
+      <c r="F34" s="20" t="n">
+        <v>77.78</v>
+      </c>
+      <c r="G34" s="20" t="n">
+        <v>75.03</v>
+      </c>
       <c r="H34" s="20" t="n"/>
       <c r="I34" s="20" t="n"/>
-      <c r="J34" s="20" t="n"/>
-      <c r="K34" s="20" t="n"/>
-      <c r="L34" s="20" t="n"/>
-      <c r="M34" s="20" t="n"/>
-      <c r="N34" s="20" t="n"/>
-      <c r="O34" s="20" t="n"/>
+      <c r="J34" s="20" t="n">
+        <v>46.94</v>
+      </c>
+      <c r="K34" s="20" t="n">
+        <v>72.01000000000001</v>
+      </c>
+      <c r="L34" s="20" t="n">
+        <v>95.06999999999999</v>
+      </c>
+      <c r="M34" s="20" t="n">
+        <v>92.23</v>
+      </c>
+      <c r="N34" s="20" t="n">
+        <v>93.73</v>
+      </c>
+      <c r="O34" s="20" t="n">
+        <v>91.81999999999999</v>
+      </c>
     </row>
     <row r="35" ht="26" customHeight="1" s="27">
       <c r="A35" s="21" t="inlineStr">
@@ -2399,18 +2787,38 @@
       <c r="C36" s="22" t="n">
         <v>2026</v>
       </c>
-      <c r="D36" s="22" t="n"/>
-      <c r="E36" s="22" t="n"/>
-      <c r="F36" s="22" t="n"/>
-      <c r="G36" s="22" t="n"/>
-      <c r="H36" s="22" t="n"/>
-      <c r="I36" s="22" t="n"/>
-      <c r="J36" s="22" t="n"/>
-      <c r="K36" s="22" t="n"/>
+      <c r="D36" s="22" t="n">
+        <v>83.11</v>
+      </c>
+      <c r="E36" s="22" t="n">
+        <v>77.06999999999999</v>
+      </c>
+      <c r="F36" s="22" t="n">
+        <v>80.66</v>
+      </c>
+      <c r="G36" s="22" t="n">
+        <v>78.33</v>
+      </c>
+      <c r="H36" s="22" t="n">
+        <v>85.67</v>
+      </c>
+      <c r="I36" s="22" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="J36" s="22" t="n">
+        <v>84.11</v>
+      </c>
+      <c r="K36" s="22" t="n">
+        <v>80.31999999999999</v>
+      </c>
       <c r="L36" s="22" t="n"/>
       <c r="M36" s="22" t="n"/>
-      <c r="N36" s="22" t="n"/>
-      <c r="O36" s="22" t="n"/>
+      <c r="N36" s="22" t="n">
+        <v>94.43000000000001</v>
+      </c>
+      <c r="O36" s="22" t="n">
+        <v>91.25</v>
+      </c>
     </row>
     <row r="37" ht="20" customHeight="1" s="27"/>
     <row r="38" ht="20" customHeight="1" s="27"/>
@@ -2843,10 +3251,18 @@
       <c r="C52" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="D52" s="20" t="n"/>
-      <c r="E52" s="20" t="n"/>
-      <c r="F52" s="20" t="n"/>
-      <c r="G52" s="20" t="n"/>
+      <c r="D52" s="20" t="n">
+        <v>84.73999999999999</v>
+      </c>
+      <c r="E52" s="20" t="n">
+        <v>76.67</v>
+      </c>
+      <c r="F52" s="20" t="n">
+        <v>80.53</v>
+      </c>
+      <c r="G52" s="20" t="n">
+        <v>76.68000000000001</v>
+      </c>
       <c r="H52" s="20" t="n">
         <v>90.23999999999999</v>
       </c>
@@ -2859,10 +3275,18 @@
       <c r="K52" s="20" t="n">
         <v>84.31999999999999</v>
       </c>
-      <c r="L52" s="20" t="n"/>
-      <c r="M52" s="20" t="n"/>
-      <c r="N52" s="20" t="n"/>
-      <c r="O52" s="20" t="n"/>
+      <c r="L52" s="20" t="n">
+        <v>58.02</v>
+      </c>
+      <c r="M52" s="20" t="n">
+        <v>45.08</v>
+      </c>
+      <c r="N52" s="20" t="n">
+        <v>50.21</v>
+      </c>
+      <c r="O52" s="20" t="n">
+        <v>44.46</v>
+      </c>
     </row>
     <row r="53" ht="17.55" customHeight="1" s="27">
       <c r="A53" s="21" t="inlineStr">
@@ -2958,8 +3382,12 @@
       </c>
       <c r="D55" s="20" t="n"/>
       <c r="E55" s="20" t="n"/>
-      <c r="F55" s="20" t="n"/>
-      <c r="G55" s="20" t="n"/>
+      <c r="F55" s="20" t="n">
+        <v>83.95999999999999</v>
+      </c>
+      <c r="G55" s="20" t="n">
+        <v>80.06999999999999</v>
+      </c>
       <c r="H55" s="20" t="n"/>
       <c r="I55" s="20" t="n"/>
       <c r="J55" s="20" t="n"/>
@@ -3465,10 +3893,18 @@
       <c r="C14" s="21" t="n">
         <v>2025</v>
       </c>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="20" t="n"/>
-      <c r="G14" s="20" t="n"/>
+      <c r="D14" s="20" t="n">
+        <v>63.47</v>
+      </c>
+      <c r="E14" s="20" t="n">
+        <v>50.05</v>
+      </c>
+      <c r="F14" s="20" t="n">
+        <v>55.33</v>
+      </c>
+      <c r="G14" s="20" t="n">
+        <v>50.08</v>
+      </c>
       <c r="H14" s="20" t="n"/>
       <c r="I14" s="20" t="n"/>
       <c r="J14" s="20" t="n"/>
@@ -3537,8 +3973,12 @@
       <c r="I16" s="20" t="n">
         <v>71.92</v>
       </c>
-      <c r="J16" s="20" t="n"/>
-      <c r="K16" s="20" t="n"/>
+      <c r="J16" s="20" t="n">
+        <v>75.73</v>
+      </c>
+      <c r="K16" s="20" t="n">
+        <v>72.64</v>
+      </c>
       <c r="L16" s="20" t="n">
         <v>86.94</v>
       </c>
@@ -4128,10 +4568,18 @@
       <c r="E35" s="20" t="n"/>
       <c r="F35" s="20" t="n"/>
       <c r="G35" s="20" t="n"/>
-      <c r="H35" s="20" t="n"/>
-      <c r="I35" s="20" t="n"/>
-      <c r="J35" s="20" t="n"/>
-      <c r="K35" s="20" t="n"/>
+      <c r="H35" s="20" t="n">
+        <v>85.36</v>
+      </c>
+      <c r="I35" s="20" t="n">
+        <v>78.75</v>
+      </c>
+      <c r="J35" s="20" t="n">
+        <v>82.17</v>
+      </c>
+      <c r="K35" s="20" t="n">
+        <v>79.05</v>
+      </c>
       <c r="L35" s="20" t="n"/>
       <c r="M35" s="20" t="n"/>
       <c r="N35" s="20" t="n"/>
@@ -4653,8 +5101,12 @@
       <c r="E54" s="20" t="n"/>
       <c r="F54" s="20" t="n"/>
       <c r="G54" s="20" t="n"/>
-      <c r="H54" s="20" t="n"/>
-      <c r="I54" s="20" t="n"/>
+      <c r="H54" s="20" t="n">
+        <v>87.56</v>
+      </c>
+      <c r="I54" s="20" t="n">
+        <v>82</v>
+      </c>
       <c r="J54" s="20" t="n"/>
       <c r="K54" s="20" t="n"/>
       <c r="L54" s="20" t="n"/>
@@ -5961,10 +6413,18 @@
       <c r="K26" s="20" t="n">
         <v>82.78</v>
       </c>
-      <c r="L26" s="20" t="n"/>
-      <c r="M26" s="20" t="n"/>
-      <c r="N26" s="20" t="n"/>
-      <c r="O26" s="20" t="n"/>
+      <c r="L26" s="20" t="n">
+        <v>98.97</v>
+      </c>
+      <c r="M26" s="20" t="n">
+        <v>97.95</v>
+      </c>
+      <c r="N26" s="20" t="n">
+        <v>49.71</v>
+      </c>
+      <c r="O26" s="20" t="n">
+        <v>97.5</v>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1" s="27">
       <c r="A27" s="21" t="inlineStr">
@@ -6004,10 +6464,18 @@
       <c r="K27" s="20" t="n">
         <v>78.23999999999999</v>
       </c>
-      <c r="L27" s="20" t="n"/>
-      <c r="M27" s="20" t="n"/>
-      <c r="N27" s="20" t="n"/>
-      <c r="O27" s="20" t="n"/>
+      <c r="L27" s="20" t="n">
+        <v>90.84</v>
+      </c>
+      <c r="M27" s="20" t="n">
+        <v>86.28</v>
+      </c>
+      <c r="N27" s="20" t="n">
+        <v>87.09</v>
+      </c>
+      <c r="O27" s="20" t="n">
+        <v>84.39</v>
+      </c>
     </row>
     <row r="28" ht="20" customHeight="1" s="27">
       <c r="A28" s="21" t="inlineStr">
@@ -6762,10 +7230,18 @@
       <c r="C45" s="21" t="n">
         <v>2023</v>
       </c>
-      <c r="D45" s="20" t="n"/>
-      <c r="E45" s="20" t="n"/>
-      <c r="F45" s="20" t="n"/>
-      <c r="G45" s="20" t="n"/>
+      <c r="D45" s="20" t="n">
+        <v>87.70999999999999</v>
+      </c>
+      <c r="E45" s="20" t="n">
+        <v>82.28</v>
+      </c>
+      <c r="F45" s="20" t="n">
+        <v>83.5</v>
+      </c>
+      <c r="G45" s="20" t="n">
+        <v>80.63</v>
+      </c>
       <c r="H45" s="20" t="n">
         <v>91.27</v>
       </c>
@@ -6778,10 +7254,18 @@
       <c r="K45" s="20" t="n">
         <v>85.63</v>
       </c>
-      <c r="L45" s="20" t="n"/>
-      <c r="M45" s="20" t="n"/>
-      <c r="N45" s="20" t="n"/>
-      <c r="O45" s="20" t="n"/>
+      <c r="L45" s="20" t="n">
+        <v>66.83</v>
+      </c>
+      <c r="M45" s="20" t="n">
+        <v>55.28</v>
+      </c>
+      <c r="N45" s="20" t="n">
+        <v>66.53</v>
+      </c>
+      <c r="O45" s="20" t="n">
+        <v>61.53</v>
+      </c>
     </row>
     <row r="46" ht="20" customHeight="1" s="27">
       <c r="A46" s="21" t="inlineStr">
@@ -6797,10 +7281,18 @@
       <c r="C46" s="21" t="n">
         <v>2023</v>
       </c>
-      <c r="D46" s="20" t="n"/>
-      <c r="E46" s="20" t="n"/>
-      <c r="F46" s="20" t="n"/>
-      <c r="G46" s="20" t="n"/>
+      <c r="D46" s="20" t="n">
+        <v>79.22</v>
+      </c>
+      <c r="E46" s="20" t="n">
+        <v>71.42</v>
+      </c>
+      <c r="F46" s="20" t="n">
+        <v>71.94</v>
+      </c>
+      <c r="G46" s="20" t="n">
+        <v>67.69</v>
+      </c>
       <c r="H46" s="20" t="n">
         <v>80.38</v>
       </c>
@@ -6813,10 +7305,18 @@
       <c r="K46" s="20" t="n">
         <v>71.55</v>
       </c>
-      <c r="L46" s="20" t="n"/>
-      <c r="M46" s="20" t="n"/>
-      <c r="N46" s="20" t="n"/>
-      <c r="O46" s="20" t="n"/>
+      <c r="L46" s="20" t="n">
+        <v>60.07</v>
+      </c>
+      <c r="M46" s="20" t="n">
+        <v>47.77</v>
+      </c>
+      <c r="N46" s="20" t="n">
+        <v>55.51</v>
+      </c>
+      <c r="O46" s="20" t="n">
+        <v>49.79</v>
+      </c>
     </row>
     <row r="47" ht="20" customHeight="1" s="27">
       <c r="A47" s="21" t="inlineStr">

</xml_diff>